<commit_message>
Derive MRIO entropy support from priors and audit staged model transitions
</commit_message>
<xml_diff>
--- a/mario/ops/cvxlab_models/Split_sectors_MRIO_KL/model_settings.xlsx
+++ b/mario/ops/cvxlab_models/Split_sectors_MRIO_KL/model_settings.xlsx
@@ -477,7 +477,7 @@
     <row r="2">
       <c r="B2" t="inlineStr">
         <is>
-          <t>Minimize(active_kl(Z_use_all,Z_use0,Zero_use_all,Reference_floor)+positive_va_kl(V,V0,Zero_V_mask,V_nonnegative_mask,Reference_floor)+free_va_kl(V_signed_positive,V_signed_negative,V0,Zero_V_mask,V_signed_mask,Reference_floor)+weighted_signed_kl(Y_all,Y0,Zero_Y_all,Weight_Y,Reference_floor)+weighted_active_kl(Z_supply_all,Z_supply0,Zero_supply_all,Weight_supply,Reference_floor))</t>
+          <t>Minimize(active_kl(Z_use_all,Z_use0,Zero_use_all,Entropy_floor)+positive_va_kl(V,V0,Zero_V_mask,V_nonnegative_mask,Entropy_floor)+free_va_kl(V_signed_positive,V_signed_negative,V0,Zero_V_mask,V_signed_mask,Entropy_floor)+weighted_signed_kl(Y_all,Y0,Zero_Y_all,Weight_Y,Entropy_floor)+weighted_active_kl(Z_supply_all,Z_supply0,Zero_supply_all,Weight_supply,Entropy_floor))</t>
         </is>
       </c>
     </row>
@@ -996,7 +996,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>parameter: [y_weight,supply_weight,reference_floor]</t>
+          <t>parameter: [y_weight,supply_weight,reference_floor,entropy_floor]</t>
         </is>
       </c>
     </row>
@@ -1011,7 +1011,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q69"/>
+  <dimension ref="A1:Q70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="12.81640625" customWidth="1" min="1" max="1"/>
@@ -3396,12 +3396,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>V_nonnegative_mask</t>
+          <t>Model_controls</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>ones where prior zeroes</t>
+          <t>Numerical model control</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -3411,37 +3411,24 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>factor, region_to, sector_to</t>
+          <t>model_control</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>V_nonnegative_mask</t>
-        </is>
-      </c>
-      <c r="H53" t="n">
-        <v>0</v>
-      </c>
-      <c r="K53" t="inlineStr">
-        <is>
-          <t>dim: cols, filters: {category: [parent, new]}</t>
-        </is>
-      </c>
-      <c r="M53" t="inlineStr">
-        <is>
-          <t>dim: cols</t>
-        </is>
-      </c>
-      <c r="O53" t="inlineStr">
-        <is>
-          <t>dim: rows</t>
+          <t>Entropy_floor</t>
+        </is>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>dim: rows, filters: {parameter: entropy_floor}</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>V_signed_mask</t>
+          <t>V_nonnegative_mask</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -3461,7 +3448,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>V_signed_mask</t>
+          <t>V_nonnegative_mask</t>
         </is>
       </c>
       <c r="H54" t="n">
@@ -3486,37 +3473,35 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>V_signed_mask</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>new final consumption</t>
+          <t>ones where prior zeroes</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>endogenous</t>
+          <t>exogenous</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>region_from, region_to, sector_from, cons_categ</t>
+          <t>factor, region_to, sector_to</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Y_all</t>
-        </is>
-      </c>
-      <c r="J55" t="inlineStr">
-        <is>
-          <t>dim: rows, filters: {category: [parent, new]}</t>
-        </is>
-      </c>
-      <c r="L55" t="inlineStr">
-        <is>
-          <t>dim: rows</t>
+          <t>V_signed_mask</t>
+        </is>
+      </c>
+      <c r="H55" t="n">
+        <v>0</v>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>dim: cols, filters: {category: [parent, new]}</t>
         </is>
       </c>
       <c r="M55" t="inlineStr">
@@ -3524,16 +3509,16 @@
           <t>dim: cols</t>
         </is>
       </c>
-      <c r="N55" t="inlineStr">
-        <is>
-          <t>dim: cols</t>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>dim: rows</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Y0</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -3543,7 +3528,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>exogenous</t>
+          <t>endogenous</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -3553,7 +3538,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Y0</t>
+          <t>Y_all</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -3580,12 +3565,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Zero_Y_mask</t>
+          <t>Y0</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>ones where prior zeroes</t>
+          <t>new final consumption</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -3600,7 +3585,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Zero_Y_all</t>
+          <t>Y0</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
@@ -3627,48 +3612,45 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Z_supply</t>
+          <t>Zero_Y_mask</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>new table of intermediate consumption supply part</t>
+          <t>ones where prior zeroes</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>endogenous</t>
+          <t>exogenous</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>region_from, region_to, sector_from, sector_to</t>
+          <t>region_from, region_to, sector_from, cons_categ</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Z_supply_all</t>
-        </is>
-      </c>
-      <c r="I58" t="b">
-        <v>1</v>
+          <t>Zero_Y_all</t>
+        </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
           <t>dim: rows, filters: {category: [parent, new]}</t>
         </is>
       </c>
-      <c r="K58" t="inlineStr">
-        <is>
-          <t>dim: cols, filters: {category: [stable]}</t>
-        </is>
-      </c>
       <c r="L58" t="inlineStr">
         <is>
           <t>dim: rows</t>
         </is>
       </c>
       <c r="M58" t="inlineStr">
+        <is>
+          <t>dim: cols</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr">
         <is>
           <t>dim: cols</t>
         </is>
@@ -3677,7 +3659,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Z_supply0</t>
+          <t>Z_supply</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -3687,7 +3669,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>exogenous</t>
+          <t>endogenous</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -3697,8 +3679,11 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Z_supply0</t>
-        </is>
+          <t>Z_supply_all</t>
+        </is>
+      </c>
+      <c r="I59" t="b">
+        <v>1</v>
       </c>
       <c r="J59" t="inlineStr">
         <is>
@@ -3724,12 +3709,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Zero_supply_mask</t>
+          <t>Z_supply0</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>ones where prior zeroes</t>
+          <t>new table of intermediate consumption supply part</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -3744,7 +3729,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Zero_supply_all</t>
+          <t>Z_supply0</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
@@ -3771,17 +3756,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Z_use</t>
+          <t>Zero_supply_mask</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>new table of intermediate consumption use part</t>
+          <t>ones where prior zeroes</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>endogenous</t>
+          <t>exogenous</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -3791,20 +3776,17 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Z_use_all</t>
-        </is>
-      </c>
-      <c r="I61" t="b">
-        <v>1</v>
+          <t>Zero_supply_all</t>
+        </is>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>dim: rows</t>
+          <t>dim: rows, filters: {category: [parent, new]}</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>dim: cols, filters: {category: [parent, new]}</t>
+          <t>dim: cols, filters: {category: [stable]}</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
@@ -3821,7 +3803,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Z_use0</t>
+          <t>Z_use</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -3831,7 +3813,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>exogenous</t>
+          <t>endogenous</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -3841,8 +3823,11 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Z_use0</t>
-        </is>
+          <t>Z_use_all</t>
+        </is>
+      </c>
+      <c r="I62" t="b">
+        <v>1</v>
       </c>
       <c r="J62" t="inlineStr">
         <is>
@@ -3868,12 +3853,12 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Zero_use_mask</t>
+          <t>Z_use0</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>ones where prior zeroes</t>
+          <t>new table of intermediate consumption use part</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -3888,7 +3873,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Zero_use_all</t>
+          <t>Z_use0</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
@@ -3915,7 +3900,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Positive_Y_mask</t>
+          <t>Zero_use_mask</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3930,20 +3915,22 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>region_from, region_to, sector_from, cons_categ</t>
+          <t>region_from, region_to, sector_from, sector_to</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Positive_Y_mask</t>
-        </is>
-      </c>
-      <c r="H64" t="n">
-        <v>0</v>
+          <t>Zero_use_all</t>
+        </is>
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>dim: rows, filters: {category: [parent, new]}</t>
+          <t>dim: rows</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>dim: cols, filters: {category: [parent, new]}</t>
         </is>
       </c>
       <c r="L64" t="inlineStr">
@@ -3952,11 +3939,6 @@
         </is>
       </c>
       <c r="M64" t="inlineStr">
-        <is>
-          <t>dim: intra</t>
-        </is>
-      </c>
-      <c r="N64" t="inlineStr">
         <is>
           <t>dim: cols</t>
         </is>
@@ -3965,7 +3947,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Negative_Y_mask</t>
+          <t>Positive_Y_mask</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3985,7 +3967,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Negative_Y_mask</t>
+          <t>Positive_Y_mask</t>
         </is>
       </c>
       <c r="H65" t="n">
@@ -4015,12 +3997,12 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>RowResidual</t>
+          <t>Negative_Y_mask</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>New total production</t>
+          <t>ones where prior zeroes</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -4030,13 +4012,16 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>region_from, sector_from</t>
+          <t>region_from, region_to, sector_from, cons_categ</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>RowResidual</t>
-        </is>
+          <t>Negative_Y_mask</t>
+        </is>
+      </c>
+      <c r="H66" t="n">
+        <v>0</v>
       </c>
       <c r="J66" t="inlineStr">
         <is>
@@ -4045,19 +4030,29 @@
       </c>
       <c r="L66" t="inlineStr">
         <is>
+          <t>dim: rows</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
           <t>dim: intra</t>
+        </is>
+      </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>dim: cols</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>ColumnResidual</t>
+          <t>RowResidual</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>New total production (r_to,s_to)</t>
+          <t>New total production</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -4067,20 +4062,20 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>region_to, sector_to</t>
+          <t>region_from, sector_from</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>ColumnResidual</t>
-        </is>
-      </c>
-      <c r="K67" t="inlineStr">
-        <is>
-          <t>dim: cols, filters: {category: [parent,new]}</t>
-        </is>
-      </c>
-      <c r="M67" t="inlineStr">
+          <t>RowResidual</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>dim: rows, filters: {category: [parent, new]}</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
         <is>
           <t>dim: intra</t>
         </is>
@@ -4089,31 +4084,28 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>V_signed_positive</t>
+          <t>ColumnResidual</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>value added row vector</t>
+          <t>New total production (r_to,s_to)</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>endogenous</t>
+          <t>exogenous</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>factor, region_to, sector_to</t>
+          <t>region_to, sector_to</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>V_signed_positive</t>
-        </is>
-      </c>
-      <c r="I68" t="b">
-        <v>1</v>
+          <t>ColumnResidual</t>
+        </is>
       </c>
       <c r="K68" t="inlineStr">
         <is>
@@ -4122,19 +4114,14 @@
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>dim: cols</t>
-        </is>
-      </c>
-      <c r="O68" t="inlineStr">
-        <is>
-          <t>dim: rows</t>
+          <t>dim: intra</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>V_signed_negative</t>
+          <t>V_signed_positive</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -4154,7 +4141,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>V_signed_negative</t>
+          <t>V_signed_positive</t>
         </is>
       </c>
       <c r="I69" t="b">
@@ -4171,6 +4158,51 @@
         </is>
       </c>
       <c r="O69" t="inlineStr">
+        <is>
+          <t>dim: rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>V_signed_negative</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>value added row vector</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>endogenous</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>factor, region_to, sector_to</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>V_signed_negative</t>
+        </is>
+      </c>
+      <c r="I70" t="b">
+        <v>1</v>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>dim: cols, filters: {category: [parent,new]}</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>dim: cols</t>
+        </is>
+      </c>
+      <c r="O70" t="inlineStr">
         <is>
           <t>dim: rows</t>
         </is>

</xml_diff>